<commit_message>
Updating H&S cia analysis
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="195" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{532A98DA-D6E0-43CA-960F-ED3174459E1D}"/>
+  <xr:revisionPtr revIDLastSave="197" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00768727-9FEF-476E-88D6-A7697251C7F2}"/>
   <bookViews>
-    <workbookView xWindow="2124" yWindow="4116" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2124" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>Royal Liverpool</t>
   </si>
@@ -127,9 +127,6 @@
   </si>
   <si>
     <t>CI going -ive, small number of falls /injuries compared to controls, some months is 0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only  5 mths data post switch, ??reported under the other Clatterbridge site code  </t>
   </si>
   <si>
     <t>CI goes negative- some months have 0 deaths</t>
@@ -615,14 +612,14 @@
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -632,17 +629,17 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="H3" s="2"/>
     </row>
@@ -669,7 +666,7 @@
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -685,7 +682,7 @@
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="3"/>
@@ -717,25 +714,23 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="2"/>
-      <c r="C9" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="C9" s="2"/>
       <c r="D9" s="4" t="s">
         <v>20</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -751,7 +746,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
       <c r="F10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -827,12 +822,12 @@
     </row>
     <row r="19" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating which sites to be included
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="197" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00768727-9FEF-476E-88D6-A7697251C7F2}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA65E63A-1910-45C3-BF24-96C07AC4988A}"/>
   <bookViews>
-    <workbookView xWindow="2124" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="972" yWindow="420" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -713,7 +713,7 @@
         <v>29</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="4" t="s">
         <v>37</v>
       </c>
       <c r="G8" s="2"/>

</xml_diff>

<commit_message>
Formatting outputs and adding summary plots
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="198" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA65E63A-1910-45C3-BF24-96C07AC4988A}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C948BC51-D7E2-4641-9223-74CBAC4AD0FF}"/>
   <bookViews>
-    <workbookView xWindow="972" yWindow="420" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1320" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>Royal Liverpool</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>Significant issues with data so don't think we can use them</t>
+  </si>
+  <si>
+    <t>Large COVID spike in outcome period.</t>
   </si>
 </sst>
 </file>
@@ -678,7 +681,7 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2" t="s">

</xml_diff>

<commit_message>
updating models with new controls
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C948BC51-D7E2-4641-9223-74CBAC4AD0FF}"/>
+  <xr:revisionPtr revIDLastSave="204" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88A101A4-2176-4BA2-864E-780BA552B8B5}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1320" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="432" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -144,9 +144,6 @@
     <t>Outcome is impacted by COVID, but so are controls, so think it might be useable</t>
   </si>
   <si>
-    <t>Controls generally have waiting lists &gt;20x larger than Clatterbridge</t>
-  </si>
-  <si>
     <t>Again controls waiting lists are generally much larger than Papworths</t>
   </si>
   <si>
@@ -166,6 +163,9 @@
   </si>
   <si>
     <t>Large COVID spike in outcome period.</t>
+  </si>
+  <si>
+    <t>CI are going -ive. Also outcome period appears to be affected by COVID increase that isn't seen in expected despite increase in control sites?</t>
   </si>
 </sst>
 </file>
@@ -619,30 +619,30 @@
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="H3" s="2"/>
     </row>
@@ -681,7 +681,7 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2" t="s">
@@ -717,7 +717,7 @@
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -825,12 +825,12 @@
     </row>
     <row r="19" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated output with new controls
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="204" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88A101A4-2176-4BA2-864E-780BA552B8B5}"/>
+  <xr:revisionPtr revIDLastSave="209" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C728F353-0A05-4685-8982-087ABF8878A5}"/>
   <bookViews>
     <workbookView xWindow="432" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -153,9 +153,6 @@
     <t>Only 4 months data in the outcome period</t>
   </si>
   <si>
-    <t>Some missing data in pre switch period, but looks like there is enough data</t>
-  </si>
-  <si>
     <t>Good!</t>
   </si>
   <si>
@@ -166,6 +163,9 @@
   </si>
   <si>
     <t>CI are going -ive. Also outcome period appears to be affected by COVID increase that isn't seen in expected despite increase in control sites?</t>
+  </si>
+  <si>
+    <t>Missing data in the 2 yr period prior to the switch, which disruptions baseline and gives -ive CIs</t>
   </si>
 </sst>
 </file>
@@ -608,7 +608,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -621,8 +621,8 @@
       <c r="F2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>38</v>
+      <c r="G2" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>35</v>
@@ -641,8 +641,8 @@
       <c r="F3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>38</v>
+      <c r="G3" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="H3" s="2"/>
     </row>
@@ -681,7 +681,7 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2" t="s">
@@ -825,12 +825,12 @@
     </row>
     <row r="19" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating CIA issues sheet
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="213" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55C115D1-0DE6-47B7-A8E9-B1849E7A04D2}"/>
+  <xr:revisionPtr revIDLastSave="227" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{543A6D83-6E2B-4FE4-A89D-6495310DFB45}"/>
   <bookViews>
-    <workbookView xWindow="432" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
   <si>
     <t>Royal Liverpool</t>
   </si>
@@ -157,16 +157,28 @@
   </si>
   <si>
     <t>Staff survey</t>
+  </si>
+  <si>
+    <t>Cleaning</t>
+  </si>
+  <si>
+    <t>Can only find one control match, and so large -ive CI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -210,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -225,6 +237,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -575,7 +594,7 @@
     <col min="10" max="10" width="20.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -598,7 +617,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -616,7 +635,7 @@
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -636,7 +655,7 @@
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -650,7 +669,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -664,7 +683,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -680,7 +699,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:8" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -694,7 +713,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -712,7 +731,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -728,12 +747,12 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="2"/>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="2"/>
@@ -744,7 +763,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -756,7 +775,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -770,30 +789,55 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="1"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="J15" s="7"/>
+    </row>
+    <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+    <row r="17" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixing plots, ordering, and updating indicator availability table
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="227" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{543A6D83-6E2B-4FE4-A89D-6495310DFB45}"/>
+  <xr:revisionPtr revIDLastSave="229" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{839BF725-7121-4C9D-88E8-3A9518CA47CD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="876" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -150,9 +150,6 @@
     <t>Large COVID spike in outcome period.</t>
   </si>
   <si>
-    <t>CI are going -ive. Also outcome period appears to be affected by COVID increase that isn't seen in expected despite increase in control sites?</t>
-  </si>
-  <si>
     <t>Missing data in the 2 yr period prior to the switch, which disruptions baseline and gives -ive CIs</t>
   </si>
   <si>
@@ -163,6 +160,9 @@
   </si>
   <si>
     <t>Can only find one control match, and so large -ive CI</t>
+  </si>
+  <si>
+    <t>Outcome period cut short due to -ive Cis as variable COVID effect.</t>
   </si>
 </sst>
 </file>
@@ -222,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -240,10 +240,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -594,7 +590,7 @@
     <col min="10" max="10" width="20.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +613,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -631,17 +627,17 @@
         <v>33</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:10" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="4" t="s">
-        <v>37</v>
+      <c r="C3" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>31</v>
@@ -651,11 +647,11 @@
         <v>33</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -669,7 +665,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -683,7 +679,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -699,7 +695,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -713,7 +709,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -731,7 +727,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -747,7 +743,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
@@ -763,7 +759,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -775,7 +771,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -789,9 +785,9 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -801,32 +797,31 @@
       <c r="G13" s="2"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="3"/>
       <c r="F14" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="J15" s="7"/>
-    </row>
-    <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>18</v>
       </c>

</xml_diff>

<commit_message>
removing Clatterbridge controls that are not purely cancer centres
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="229" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{839BF725-7121-4C9D-88E8-3A9518CA47CD}"/>
+  <xr:revisionPtr revIDLastSave="258" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1228969-9C22-46B5-9037-246CA9B795DB}"/>
   <bookViews>
-    <workbookView xWindow="876" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5772" yWindow="7320" windowWidth="20160" windowHeight="13800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t>Royal Liverpool</t>
   </si>
@@ -163,6 +163,48 @@
   </si>
   <si>
     <t>Outcome period cut short due to -ive Cis as variable COVID effect.</t>
+  </si>
+  <si>
+    <t>HCAI</t>
+  </si>
+  <si>
+    <t>c.diff</t>
+  </si>
+  <si>
+    <t>e.coli</t>
+  </si>
+  <si>
+    <t>remove from combined</t>
+  </si>
+  <si>
+    <t>Klebsiella</t>
+  </si>
+  <si>
+    <t>mrsa</t>
+  </si>
+  <si>
+    <t>mssa</t>
+  </si>
+  <si>
+    <t>p.aerurinosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UDAL data availability </t>
+  </si>
+  <si>
+    <t>Archive</t>
+  </si>
+  <si>
+    <t>Only back to 2017</t>
+  </si>
+  <si>
+    <t>Goes to 2016, but only at regional not provider level</t>
+  </si>
+  <si>
+    <t>Combined measure can go back to March 2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Even if you drop e.coli and mrsa then for combined data you can only go back to April 2017 which is still less than 2 years baseline for Papworth </t>
   </si>
 </sst>
 </file>
@@ -222,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -240,6 +282,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -843,12 +886,100 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0E9BC20-D7AB-46BB-901F-6A9F26AEA7B1}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" customWidth="1"/>
+    <col min="2" max="3" width="18.109375" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="7">
+        <v>41000</v>
+      </c>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="7">
+        <v>43160</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="7">
+        <v>42826</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="7">
+        <v>43160</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="7">
+        <v>42826</v>
+      </c>
+      <c r="C6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="7">
+        <v>42826</v>
+      </c>
+      <c r="C7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Adding c.diff as indicator variable
</commit_message>
<xml_diff>
--- a/CIA issues.xlsx
+++ b/CIA issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/sarah_lucas3_nhs_net/Documents/Documents/NHP Single Bed Accomodation/NHP Single Bed Room/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="258" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1228969-9C22-46B5-9037-246CA9B795DB}"/>
+  <xr:revisionPtr revIDLastSave="276" documentId="10_ncr:40000_{7B144F86-E0FF-4ED7-A1CE-E205DB84DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AB4EBBD-BD8D-4805-958D-5BDB7153A1CC}"/>
   <bookViews>
-    <workbookView xWindow="5772" yWindow="7320" windowWidth="20160" windowHeight="13800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20160" windowHeight="13800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="57">
   <si>
     <t>Royal Liverpool</t>
   </si>
@@ -201,10 +201,13 @@
     <t>Goes to 2016, but only at regional not provider level</t>
   </si>
   <si>
-    <t>Combined measure can go back to March 2018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Even if you drop e.coli and mrsa then for combined data you can only go back to April 2017 which is still less than 2 years baseline for Papworth </t>
+    <t>C.difficile</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Rates are very low, lots of zeros, even summing cases annually get -ive Cis</t>
   </si>
 </sst>
 </file>
@@ -624,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -752,130 +755,152 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="4" t="s">
+      <c r="B9" s="2"/>
+      <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="4" t="s">
-        <v>20</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2" t="s">
+      <c r="B11" s="2"/>
+      <c r="C11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="4" t="s">
+      <c r="E14" s="6"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+    <row r="18" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
         <v>34</v>
       </c>
     </row>
@@ -886,7 +911,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0E9BC20-D7AB-46BB-901F-6A9F26AEA7B1}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" customWidth="1"/>
@@ -967,16 +992,6 @@
       </c>
       <c r="C7" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>